<commit_message>
Crawl: widen scope from a leaf start page; skip translations
Unreal Engine's docs landing page (.../unreal-engine-5-8-documentation)
has no trailing slash and links only to siblings, so the crawl found one
page. When the start page is a leaf with nothing in scope, move the bound
up one folder (never to the site root). Skip ?lang=/hl=/locale= copies.

Inventory D0172 now uses the locale-free /documentation/unreal-engine/
path that the site's own links use.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S3bpT6u3Lki3dEMTGSRFRc
</commit_message>
<xml_diff>
--- a/inventory/swarm-technology-document-inventory.xlsx
+++ b/inventory/swarm-technology-document-inventory.xlsx
@@ -22197,7 +22197,7 @@
       </c>
       <c r="E173" s="25" t="inlineStr">
         <is>
-          <t>https://dev.epicgames.com/documentation/en-us/unreal-engine</t>
+          <t>https://dev.epicgames.com/documentation/unreal-engine/</t>
         </is>
       </c>
       <c r="F173" s="16" t="inlineStr">
@@ -22223,12 +22223,12 @@
       </c>
       <c r="K173" s="16" t="inlineStr">
         <is>
-          <t>From general knowledge, not seen this session (confirm before scraping)</t>
+          <t>Checked live on 22 September 2026 (URL corrected)</t>
         </is>
       </c>
       <c r="L173" s="16" t="inlineStr">
         <is>
-          <t>Very large; scrape only if AirSim-family work goes ahead.</t>
+          <t>Very large; scrape only if AirSim-family work goes ahead. URL corrected after live test: the en-us path redirects to a page whose links all use the locale-free /documentation/unreal-engine/ path (was https://dev.epicgames.com/documentation/en-us/unreal-engine).</t>
         </is>
       </c>
     </row>

</xml_diff>